<commit_message>
enrich modifié, nouveau prog.json
</commit_message>
<xml_diff>
--- a/Lab/outils/work/enriched.xlsx
+++ b/Lab/outils/work/enriched.xlsx
@@ -601,7 +601,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>United Kingdom, United States of America</t>
+          <t>Grande-Bretagne</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -801,7 +801,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Morocco, France, Spain, Germany, Belgium</t>
+          <t>France, Espagne, Maroc, Allemagne, Belgique</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -875,10 +875,14 @@
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://fr.web.img3.acsta.net/c_310_420/medias/nmedia/18/70/18/27/19090499.jpg</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Voyage sur terre à l’échelle du centimètre. Ses habitants: insectes et autres animaux de l'herbe et de l'eau. Grand prix de la commission supérieure technique, Festival de Cannes 1996.</t>
+          <t>Voyage sur terre à l'echelle du centimètre. Ses habitants: insectes et autres animaux de l'herbe et de l'eau. Grand prix de la commission supérieure technique, Festival de Cannes 1996.</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -893,7 +897,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>France, Switzerland, Italy</t>
+          <t>France, Suisse, Italie</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -901,10 +905,14 @@
           <t>Jacques Perrin</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>2.8, César 1997: César de la Meilleure musique écrite pour un film, César du Producteur de l'année, César du Meilleur montage, César de la Meilleure photographie, César du Meilleur son, Festival de Cannes 1996: Prix Vulcain de l'Artiste-Technicien, Fondation Gan pour le cinéma 1992: Prix Fondation Gan</t>
+        </is>
+      </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1996-05-20</t>
+          <t>1996-11-20</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -912,11 +920,19 @@
           <t>https://www.youtube.com/watch?v=5fA3h9dy1NQ</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=42006.html</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>["https://fr.web.img2.acsta.net/medias/nmedia/18/70/18/27/19090502.jpg", "https://fr.web.img6.acsta.net/medias/nmedia/18/70/18/27/19090501.jpg", "https://fr.web.img3.acsta.net/medias/nmedia/18/70/18/27/19090503.jpg", "https://fr.web.img4.acsta.net/medias/nmedia/18/70/18/27/19090504.jpg", "https://fr.web.img5.acsta.net/medias/nmedia/18/70/18/27/19090505.jpg"]</t>
+        </is>
+      </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>1996-05-20</t>
+          <t>1996-11-20</t>
         </is>
       </c>
     </row>
@@ -1055,7 +1071,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Cinélatino Avant-première</t>
+          <t>Cinélatino Avant - première</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
@@ -1081,7 +1097,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Colombia, Brazil, France</t>
+          <t>France, Colombie, Brésil</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1099,7 +1115,11 @@
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr"/>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>https://www.allocine.fr/video/player_gen_cmedia=20633447&amp;cfilm=325278.html</t>
+        </is>
+      </c>
       <c r="T7" t="inlineStr">
         <is>
           <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=325278.html</t>
@@ -1165,7 +1185,7 @@
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>France, Russie</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -1179,7 +1199,11 @@
           <t>2026-02-18</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr"/>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>https://www.allocine.fr/video/player_gen_cmedia=20630887&amp;cfilm=1000031821.html</t>
+        </is>
+      </c>
       <c r="T8" t="inlineStr">
         <is>
           <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000031821.html</t>
@@ -1235,7 +1259,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Ciné Documentaire du samedi 18h</t>
+          <t>Ciné Documentaire du samedi 18 €h</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -1361,7 +1385,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>United States of America</t>
+          <t>U.S.A.</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1461,7 +1485,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>France, Belgium</t>
+          <t>France</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -1549,7 +1573,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>France, Belgium</t>
+          <t>France, Belgique</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1645,7 +1669,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Germany, United Kingdom</t>
+          <t>Grande-Bretagne</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -1737,7 +1761,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>France, United States of America</t>
+          <t>France, U.S.A.</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -1849,7 +1873,11 @@
           <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000023077.html</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr"/>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>["https://image.tmdb.org/t/p/original/jwFj1fIxffU6CziBoufDiqNrkKA.jpg"]</t>
+        </is>
+      </c>
       <c r="V15" t="inlineStr">
         <is>
           <t>2026-03-04</t>
@@ -1913,7 +1941,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Croatia, Slovenia, Serbia, Italy</t>
+          <t>Slovénie, Italie, Croatie, Serbie</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -2009,7 +2037,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>United States of America</t>
+          <t>U.S.A.</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -2087,25 +2115,29 @@
       </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>https://fr.web.img4.acsta.net/c_310_420/img/cb/92/cb92cf130cfc390336b1400c7130de6f.jpg</t>
+        </is>
+      </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Ex-membre des marines, Louanne Johnson accepte d'enseigner à la East Palo Alto Highschool, un établissement à la réputation sulfureuse. Réalisant que ses élèves possèdent de grandes capacités intellectuelles, elle décide de se battre pour les aider à apprendre.</t>
+          <t>Un tournesol hors norme, un gnome déterminé, une petite fille intrépide, défiant les lois de la nature, une fourmi rêveuse, des créatures gloutonnes… nul doute, la rébellion est en marche ! Programme de 6 courts métrages.Programme de 6 courts métrages : - Tournesol de Natalia Chernysheva (France, 2023, 4') : Un tournesol pas comme les autres choisit deporter un regard nouveau sur son environnement, il va découvrir un univers totalement différent…- Le Renard minuscule de Sylwia Szkiladz et Aline Quertain (Belgique, France, Suisse, 2015, 8') : Au milieu d'un jardin foisonnant, un tout petit renard rencontre une enfant intrépide qui fait pousser des plantes géantes ! Par un joyeux hasard, ils découvrent qu’ils peuvent faire pousser des objets, cela va donner des idées aux petits malins…- La Marche des fourmis de Fedor Yudin (Russie, 2022, 5') : Une fourmi part à la découverte du monde qui l'entoure et explore ses richesses sonores et musicales. Inspiré de l'art graphique chinois, ce film musical propose une contemplation de la nature et attire l'attention sur la beauté des choses petites et simples.- Le Gnome et le Nuage de Zuzana Čupová et Filip Diviak (République Tchèque, 2019, 5') : Petite île, ciel radieux. Monsieur Gnome souhaite passer cette splendide journée à bronzer sur un transat. Un petit nuage se met juste devant le soleil, ne lui laissant pas le temps d’en profiter. Mais Monsieur Gnome sait exactement quoi faire !- Le Dragon et la musique de Camille Muller (Suisse, 2015, 8') : L'amitié d'une petite joueuse de flûte et d'un dragon mélomane au sein d'un royaume n'autorisant que les marches militaires.- Mojappi - C'est à moi de Nijitaro (Japon, 2025, 3') : Dans la forêt, trois petites créatures fort coquines convoitent le gros pancake que se préparent leurs camarades. Tous les stratagèmes sont bons pour le récupérer !</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Drame</t>
+          <t>Animation, Famille</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>34</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>United States of America</t>
+          <t>France, Belgique, Suisse, Russie, République tchèque, Japon</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -2113,10 +2145,14 @@
           <t>Michelle Pfeiffer, George Dzundza, Courtney B. Vance, Robin Bartlett, Beatrice Winde, John Neville, Lorraine Toussaint, Renoly Santiago</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>TU 3 €</t>
+        </is>
+      </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1996-02-07</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2124,11 +2160,19 @@
           <t>https://www.youtube.com/watch?v=gA-5nLQCmW8</t>
         </is>
       </c>
-      <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000036350.html</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>["https://fr.web.img5.acsta.net/img/4d/3c/4d3c7c4e51dcbb9c80ffa5db14a73afc.jpg", "https://fr.web.img4.acsta.net/img/aa/e1/aae1206b0311fb98aa0b613fd0cae29c.jpg", "https://fr.web.img3.acsta.net/img/85/77/8577949b432f39a0ab74c42315116e98.jpg", "https://fr.web.img6.acsta.net/img/7e/68/7e68d676372286e18b74e70be35e2ed4.jpg", "https://fr.web.img6.acsta.net/img/bf/48/bf482ae0bc64f3b584ef51abfc49aa15.jpg", "https://fr.web.img4.acsta.net/img/9e/ce/9ece6ddec5938f58bfa666c3b93958aa.jpg"]</t>
+        </is>
+      </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>1996-02-07</t>
+          <t>2026-02-18</t>
         </is>
       </c>
     </row>
@@ -2167,7 +2211,7 @@
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Ciné Patrimoine du samedi 18h</t>
+          <t>Ciné Patrimoine du samedi 18 €h</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
@@ -2193,7 +2237,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Hong-Kong</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -2285,7 +2329,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>France, Canada</t>
+          <t>France</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -2477,7 +2521,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>France, Belgium</t>
+          <t>France</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -2565,7 +2609,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Belgium, France</t>
+          <t>France, Belgique</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -2661,7 +2705,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>France, Belgium</t>
+          <t>France</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -2845,7 +2889,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Allemagne</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -2937,7 +2981,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Germany, Cyprus, United States of America, Qatar, Saudi Arabia, Egypt, United Arab Emirates, Jordan, Kuwait</t>
+          <t>Allemagne, Chypre, Palestine, U.S.A., Jordanie, Emirats Arabes Unis</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -3033,7 +3077,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>France, Canada</t>
+          <t>France</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
@@ -3129,7 +3173,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Lebanon, United States of America, Germany, Greece</t>
+          <t>Liban, U.S.A., Allemagne, Arabie Saoudite, Qatar</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -3229,7 +3273,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>United States of America</t>
+          <t>U.S.A.</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -3303,7 +3347,7 @@
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Ciné Jeunes du samedi 18h</t>
+          <t>Ciné Jeunes du samedi 18 €h</t>
         </is>
       </c>
       <c r="J31" t="inlineStr"/>
@@ -3329,7 +3373,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>United States of America</t>
+          <t>U.S.A.</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
@@ -3491,7 +3535,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Famille  à partir de 9/10 ans</t>
+          <t>Famille à partir de 9 € / 10 ans</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -3521,7 +3565,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>France, Luxembourg, Canada, Belgium</t>
+          <t>France, Luxembourg, Canada, Belgique</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
@@ -3785,7 +3829,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>France, Canada</t>
+          <t>France</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
@@ -3881,7 +3925,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>United States of America</t>
+          <t>U.S.A.</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
@@ -3955,18 +3999,58 @@
         </is>
       </c>
       <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
-      <c r="O38" t="inlineStr"/>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>https://fr.web.img6.acsta.net/c_310_420/img/48/5a/485af2a4575500546e6af0c462d9f150.jpg</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Mahnaz, une infirmière de 45 ans, élève seule ses enfants. Alors qu’elle s’apprête à épouser son petit ami Hamid, son fils Aliyar est renvoyé de l’école. Lorsqu’un un accident tragique vient tout bouleverser, Mahnaz se lance dans une quête de justice pour obtenir réparation...</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>Drame</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>131</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Iran</t>
+        </is>
+      </c>
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
-      <c r="R38" t="inlineStr"/>
-      <c r="S38" t="inlineStr"/>
-      <c r="T38" t="inlineStr"/>
-      <c r="U38" t="inlineStr"/>
-      <c r="V38" t="inlineStr"/>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>https://www.allocine.fr/video/player_gen_cmedia=20632702&amp;cfilm=1000019745.html</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>https://www.allocine.fr/film/fichefilm_gen_cfilm=1000019745.html</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>["https://fr.web.img5.acsta.net/img/42/20/4220d60b7edb1ed8c0b8a85ea8ad9582.jpg", "https://fr.web.img4.acsta.net/img/77/a1/77a1bde1cabfd2b837735ac3a1c9ff72.jpg", "https://fr.web.img5.acsta.net/img/a4/b2/a4b2a9aa5fcbb8581be337ff35ce644b.jpg", "https://fr.web.img6.acsta.net/img/30/f6/30f6c8d983f12011d6edfbca88b118e1.jpg", "https://fr.web.img2.acsta.net/img/b6/8f/b68ff068e5eefbfad3c6393a1d1cd6f5.jpg", "https://fr.web.img4.acsta.net/img/b1/54/b1545b5f632dfd513dcf79312f5deda3.jpg", "https://fr.web.img5.acsta.net/img/50/69/5069460ce8637aff4292a0f24b5744d1.jpg"]</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4025,7 +4109,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>United Kingdom, Ireland, Netherlands</t>
+          <t>Grande-Bretagne, Irlande</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
@@ -4125,7 +4209,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>Ireland, Luxembourg, Belgium, Denmark</t>
+          <t>Irlande, Danemark, Belgique, Luxembourg, France</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
@@ -4221,7 +4305,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>Japan, France</t>
+          <t>Japon, France</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
@@ -4309,7 +4393,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Italie</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
@@ -4379,7 +4463,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>ados à partir de 9/10 ans Sony</t>
+          <t>ados à partir de 9 € / 10 ans Sony</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -4409,7 +4493,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Japon, U.S.A.</t>
         </is>
       </c>
       <c r="P43" t="inlineStr">
@@ -4479,7 +4563,7 @@
       <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Ciné Discussion du samedi 18h</t>
+          <t>Ciné Discussion du samedi 18 €h</t>
         </is>
       </c>
       <c r="J44" t="inlineStr"/>
@@ -4505,7 +4589,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Italie</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
@@ -4601,7 +4685,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>United Kingdom, United States of America, Sweden</t>
+          <t>U.S.A.</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
@@ -4701,7 +4785,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>Belgium, France</t>
+          <t>France, Belgique</t>
         </is>
       </c>
       <c r="P46" t="inlineStr"/>
@@ -4885,7 +4969,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>France, Ireland, United States of America, United Kingdom</t>
+          <t>Irlande, U.S.A.</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -4985,7 +5069,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>France, Ireland, United States of America, United Kingdom</t>
+          <t>Irlande, U.S.A.</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -5081,7 +5165,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>Belgium, France</t>
+          <t>Belgique, France</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">

</xml_diff>